<commit_message>
Biblioteca: 16 fuentes nuevas de sanidad y economía (974 registros)
</commit_message>
<xml_diff>
--- a/biblioteca_canamo_siccan.xlsx
+++ b/biblioteca_canamo_siccan.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Registros'!$A$1:$L$959</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Registros'!$A$1:$L$975</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,13 @@
       <color rgb="002F5D50"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -96,10 +103,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,9 +136,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -617,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -720,6 +730,13 @@
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Cómo citar: SICCAN (2026). Biblioteca Cáñamo SICCAN: registros de la revisión sistemática [Base de datos]. Universidad Nacional de Colombia, Sede Palmira.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Actualización 14/10/2026: se agregaron 16 fuentes de una búsqueda dirigida sobre sanidad (plagas, enfermedades, Fusarium, Pythium, MIPE, control biológico) y economía (costos, sistema agroecológico frente a convencional), con el tema nuevo "Sanidad: plagas y enfermedades". Las fuentes usadas en el artículo (versión 9) están marcadas con "Sí" y resaltadas.</t>
         </is>
       </c>
     </row>
@@ -734,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L959"/>
+  <dimension ref="A1:L975"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8788,54 +8805,58 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="5" t="n">
+      <c r="A151" s="8" t="n">
         <v>2025</v>
       </c>
-      <c r="B151" s="6" t="inlineStr">
+      <c r="B151" s="9" t="inlineStr">
         <is>
           <t>Sex Expression and Seed Yield Stability in Thai Hemp (Cannabis sativa L.): Seasonal Effects on Dioecious Cultivars for Optimized Seed Production</t>
         </is>
       </c>
-      <c r="C151" s="6" t="inlineStr">
+      <c r="C151" s="9" t="inlineStr">
         <is>
           <t>International Journal of Plant Biology</t>
         </is>
       </c>
-      <c r="D151" s="5" t="inlineStr">
+      <c r="D151" s="8" t="inlineStr">
         <is>
           <t>TH</t>
         </is>
       </c>
-      <c r="E151" s="6" t="inlineStr">
+      <c r="E151" s="9" t="inlineStr">
         <is>
           <t>Grano y semilla; Trópico y países de baja latitud; Cultivares y tipos de cultivo</t>
         </is>
       </c>
-      <c r="F151" s="6" t="inlineStr">
+      <c r="F151" s="9" t="inlineStr">
         <is>
           <t>Agronomía de grano</t>
         </is>
       </c>
-      <c r="G151" s="5" t="n">
+      <c r="G151" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H151" s="5" t="inlineStr">
+      <c r="H151" s="8" t="inlineStr">
         <is>
           <t>Abierto (oro/verde)</t>
         </is>
       </c>
-      <c r="I151" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J151" s="5" t="inlineStr"/>
-      <c r="K151" s="7" t="inlineStr">
+      <c r="I151" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J151" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K151" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/ijpb16020067</t>
         </is>
       </c>
-      <c r="L151" s="7" t="inlineStr">
+      <c r="L151" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W4411283630</t>
         </is>
@@ -9536,54 +9557,58 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="5" t="n">
+      <c r="A165" s="8" t="n">
         <v>2025</v>
       </c>
-      <c r="B165" s="6" t="inlineStr">
+      <c r="B165" s="9" t="inlineStr">
         <is>
           <t>Economic feasibility and risk analysis of industrial hemp production: a comparative assessment of floral, fiber, and grain enterprises in North Carolina, USA</t>
         </is>
       </c>
-      <c r="C165" s="6" t="inlineStr">
+      <c r="C165" s="9" t="inlineStr">
         <is>
           <t>Journal of Cannabis Research</t>
         </is>
       </c>
-      <c r="D165" s="5" t="inlineStr">
+      <c r="D165" s="8" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E165" s="6" t="inlineStr">
+      <c r="E165" s="9" t="inlineStr">
         <is>
           <t>Grano y semilla; Mercado y economía; Cultivares y tipos de cultivo</t>
         </is>
       </c>
-      <c r="F165" s="6" t="inlineStr">
+      <c r="F165" s="9" t="inlineStr">
         <is>
           <t>Agronomía de grano; Mercado</t>
         </is>
       </c>
-      <c r="G165" s="5" t="n">
+      <c r="G165" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H165" s="5" t="inlineStr">
+      <c r="H165" s="8" t="inlineStr">
         <is>
           <t>Abierto (oro/verde)</t>
         </is>
       </c>
-      <c r="I165" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J165" s="5" t="inlineStr"/>
-      <c r="K165" s="7" t="inlineStr">
+      <c r="I165" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J165" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K165" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.1186/s42238-025-00364-x</t>
         </is>
       </c>
-      <c r="L165" s="7" t="inlineStr">
+      <c r="L165" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W4417107606</t>
         </is>
@@ -14450,54 +14475,58 @@
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="5" t="n">
+      <c r="A258" s="8" t="n">
         <v>2024</v>
       </c>
-      <c r="B258" s="6" t="inlineStr">
+      <c r="B258" s="9" t="inlineStr">
         <is>
           <t>A FLOWERING LOCUS T ortholog is associated with photoperiod‐insensitive flowering in hemp (Cannabis sativa L.)</t>
         </is>
       </c>
-      <c r="C258" s="6" t="inlineStr">
+      <c r="C258" s="9" t="inlineStr">
         <is>
           <t>The Plant Journal</t>
         </is>
       </c>
-      <c r="D258" s="5" t="inlineStr">
+      <c r="D258" s="8" t="inlineStr">
         <is>
           <t>IE; US</t>
         </is>
       </c>
-      <c r="E258" s="6" t="inlineStr">
+      <c r="E258" s="9" t="inlineStr">
         <is>
           <t>Fenología y floración</t>
         </is>
       </c>
-      <c r="F258" s="6" t="inlineStr">
+      <c r="F258" s="9" t="inlineStr">
         <is>
           <t>Fenología y fotoperiodo</t>
         </is>
       </c>
-      <c r="G258" s="5" t="n">
+      <c r="G258" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="H258" s="5" t="inlineStr">
+      <c r="H258" s="8" t="inlineStr">
         <is>
           <t>Abierto (híbrido)</t>
         </is>
       </c>
-      <c r="I258" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J258" s="5" t="inlineStr"/>
-      <c r="K258" s="7" t="inlineStr">
+      <c r="I258" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J258" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K258" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/tpj.16769</t>
         </is>
       </c>
-      <c r="L258" s="7" t="inlineStr">
+      <c r="L258" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W4394856039</t>
         </is>
@@ -23484,54 +23513,58 @@
       </c>
     </row>
     <row r="427">
-      <c r="A427" s="5" t="n">
+      <c r="A427" s="8" t="n">
         <v>2023</v>
       </c>
-      <c r="B427" s="6" t="inlineStr">
+      <c r="B427" s="9" t="inlineStr">
         <is>
           <t>Qualitative Analysis of Industrial Hemp Production, Markets, and Sustainability in North Carolina, United States</t>
         </is>
       </c>
-      <c r="C427" s="6" t="inlineStr">
+      <c r="C427" s="9" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="D427" s="5" t="inlineStr">
+      <c r="D427" s="8" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E427" s="6" t="inlineStr">
+      <c r="E427" s="9" t="inlineStr">
         <is>
           <t>Mercado y economía</t>
         </is>
       </c>
-      <c r="F427" s="6" t="inlineStr">
+      <c r="F427" s="9" t="inlineStr">
         <is>
           <t>Mercado; Productores, asociatividad y mano de obra</t>
         </is>
       </c>
-      <c r="G427" s="5" t="n">
+      <c r="G427" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="H427" s="5" t="inlineStr">
+      <c r="H427" s="8" t="inlineStr">
         <is>
           <t>Abierto (oro/verde)</t>
         </is>
       </c>
-      <c r="I427" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J427" s="5" t="inlineStr"/>
-      <c r="K427" s="7" t="inlineStr">
+      <c r="I427" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J427" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K427" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/agriculture13040887</t>
         </is>
       </c>
-      <c r="L427" s="7" t="inlineStr">
+      <c r="L427" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W4366348945</t>
         </is>
@@ -27678,54 +27711,58 @@
       </c>
     </row>
     <row r="506">
-      <c r="A506" s="5" t="n">
+      <c r="A506" s="8" t="n">
         <v>2022</v>
       </c>
-      <c r="B506" s="6" t="inlineStr">
+      <c r="B506" s="9" t="inlineStr">
         <is>
           <t>The cannabinoid profile and growth of hemp (Cannabis sativa L.) is influenced by tropical daylengths and temperatures, genotype and nitrogen nutrition</t>
         </is>
       </c>
-      <c r="C506" s="6" t="inlineStr">
+      <c r="C506" s="9" t="inlineStr">
         <is>
           <t>Industrial Crops and Products</t>
         </is>
       </c>
-      <c r="D506" s="5" t="inlineStr">
+      <c r="D506" s="8" t="inlineStr">
         <is>
           <t>AU</t>
         </is>
       </c>
-      <c r="E506" s="6" t="inlineStr">
+      <c r="E506" s="9" t="inlineStr">
         <is>
           <t>Nutrición y fertilización; Trópico y países de baja latitud; Cultivares y tipos de cultivo</t>
         </is>
       </c>
-      <c r="F506" s="6" t="inlineStr">
+      <c r="F506" s="9" t="inlineStr">
         <is>
           <t>Trópico y Colombia</t>
         </is>
       </c>
-      <c r="G506" s="5" t="n">
+      <c r="G506" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="H506" s="5" t="inlineStr">
+      <c r="H506" s="8" t="inlineStr">
         <is>
           <t>Cerrado</t>
         </is>
       </c>
-      <c r="I506" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J506" s="5" t="inlineStr"/>
-      <c r="K506" s="7" t="inlineStr">
+      <c r="I506" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J506" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K506" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.indcrop.2022.114605</t>
         </is>
       </c>
-      <c r="L506" s="7" t="inlineStr">
+      <c r="L506" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W4210952993</t>
         </is>
@@ -28268,54 +28305,58 @@
       </c>
     </row>
     <row r="517">
-      <c r="A517" s="5" t="n">
+      <c r="A517" s="8" t="n">
         <v>2022</v>
       </c>
-      <c r="B517" s="6" t="inlineStr">
+      <c r="B517" s="9" t="inlineStr">
         <is>
           <t>Identification and mapping of major-effect flowering time loci Autoflower1 and Early1 in Cannabis sativa L.</t>
         </is>
       </c>
-      <c r="C517" s="6" t="inlineStr">
+      <c r="C517" s="9" t="inlineStr">
         <is>
           <t>Frontiers in Plant Science</t>
         </is>
       </c>
-      <c r="D517" s="5" t="inlineStr">
+      <c r="D517" s="8" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E517" s="6" t="inlineStr">
+      <c r="E517" s="9" t="inlineStr">
         <is>
           <t>Fenología y floración</t>
         </is>
       </c>
-      <c r="F517" s="6" t="inlineStr">
+      <c r="F517" s="9" t="inlineStr">
         <is>
           <t>Agronomía de grano; Fenología y fotoperiodo</t>
         </is>
       </c>
-      <c r="G517" s="5" t="n">
+      <c r="G517" s="8" t="n">
         <v>33</v>
       </c>
-      <c r="H517" s="5" t="inlineStr">
+      <c r="H517" s="8" t="inlineStr">
         <is>
           <t>Abierto (oro/verde)</t>
         </is>
       </c>
-      <c r="I517" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J517" s="5" t="inlineStr"/>
-      <c r="K517" s="7" t="inlineStr">
+      <c r="I517" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J517" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K517" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.3389/fpls.2022.991680</t>
         </is>
       </c>
-      <c r="L517" s="7" t="inlineStr">
+      <c r="L517" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W4297878948</t>
         </is>
@@ -30886,54 +30927,58 @@
       </c>
     </row>
     <row r="566">
-      <c r="A566" s="5" t="n">
+      <c r="A566" s="8" t="n">
         <v>2022</v>
       </c>
-      <c r="B566" s="6" t="inlineStr">
+      <c r="B566" s="9" t="inlineStr">
         <is>
           <t>Identificación de microorganismos asociados al suelo, sustrato y agua de un sistema productivo de Cannabis sativa L.</t>
         </is>
       </c>
-      <c r="C566" s="6" t="inlineStr">
+      <c r="C566" s="9" t="inlineStr">
         <is>
           <t>Temas Agrarios</t>
         </is>
       </c>
-      <c r="D566" s="5" t="inlineStr">
+      <c r="D566" s="8" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="E566" s="6" t="inlineStr">
+      <c r="E566" s="9" t="inlineStr">
         <is>
           <t>Suelo</t>
         </is>
       </c>
-      <c r="F566" s="6" t="inlineStr">
+      <c r="F566" s="9" t="inlineStr">
         <is>
           <t>Trópico y Colombia; Literatura en español</t>
         </is>
       </c>
-      <c r="G566" s="5" t="n">
+      <c r="G566" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H566" s="5" t="inlineStr">
+      <c r="H566" s="8" t="inlineStr">
         <is>
           <t>Abierto (diamante)</t>
         </is>
       </c>
-      <c r="I566" s="5" t="inlineStr">
+      <c r="I566" s="8" t="inlineStr">
         <is>
           <t>Español</t>
         </is>
       </c>
-      <c r="J566" s="5" t="inlineStr"/>
-      <c r="K566" s="7" t="inlineStr">
+      <c r="J566" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K566" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.21897/rta.v27i1.3111</t>
         </is>
       </c>
-      <c r="L566" s="7" t="inlineStr">
+      <c r="L566" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W4313512106</t>
         </is>
@@ -35520,54 +35565,58 @@
       </c>
     </row>
     <row r="653">
-      <c r="A653" s="5" t="n">
+      <c r="A653" s="8" t="n">
         <v>2021</v>
       </c>
-      <c r="B653" s="6" t="inlineStr">
+      <c r="B653" s="9" t="inlineStr">
         <is>
           <t>Response of hemp (Cannabis sativa L.) to integrated application of chemical and manure fertilizers</t>
         </is>
       </c>
-      <c r="C653" s="6" t="inlineStr">
+      <c r="C653" s="9" t="inlineStr">
         <is>
           <t>Acta agriculturae Slovenica</t>
         </is>
       </c>
-      <c r="D653" s="5" t="inlineStr">
+      <c r="D653" s="8" t="inlineStr">
         <is>
           <t>IR</t>
         </is>
       </c>
-      <c r="E653" s="6" t="inlineStr">
+      <c r="E653" s="9" t="inlineStr">
         <is>
           <t>Nutrición y fertilización</t>
         </is>
       </c>
-      <c r="F653" s="6" t="inlineStr">
+      <c r="F653" s="9" t="inlineStr">
         <is>
           <t>Agronomía de grano; Suelo y encalado</t>
         </is>
       </c>
-      <c r="G653" s="5" t="n">
+      <c r="G653" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="H653" s="5" t="inlineStr">
+      <c r="H653" s="8" t="inlineStr">
         <is>
           <t>Abierto (diamante)</t>
         </is>
       </c>
-      <c r="I653" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J653" s="5" t="inlineStr"/>
-      <c r="K653" s="7" t="inlineStr">
+      <c r="I653" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J653" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K653" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.14720/aas.2021.117.2.1819</t>
         </is>
       </c>
-      <c r="L653" s="7" t="inlineStr">
+      <c r="L653" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W3183065912</t>
         </is>
@@ -38426,54 +38475,58 @@
       </c>
     </row>
     <row r="708">
-      <c r="A708" s="5" t="n">
+      <c r="A708" s="8" t="n">
         <v>2020</v>
       </c>
-      <c r="B708" s="6" t="inlineStr">
+      <c r="B708" s="9" t="inlineStr">
         <is>
           <t>Silicon‐induced mitigatory effects in salt‐stressed hemp leaves</t>
         </is>
       </c>
-      <c r="C708" s="6" t="inlineStr">
+      <c r="C708" s="9" t="inlineStr">
         <is>
           <t>Physiologia Plantarum</t>
         </is>
       </c>
-      <c r="D708" s="5" t="inlineStr">
+      <c r="D708" s="8" t="inlineStr">
         <is>
           <t>IT; IN; LU</t>
         </is>
       </c>
-      <c r="E708" s="6" t="inlineStr">
+      <c r="E708" s="9" t="inlineStr">
         <is>
           <t>Nutrición y fertilización</t>
         </is>
       </c>
-      <c r="F708" s="6" t="inlineStr">
+      <c r="F708" s="9" t="inlineStr">
         <is>
           <t>B, Mn, Si y análisis de tejido</t>
         </is>
       </c>
-      <c r="G708" s="5" t="n">
+      <c r="G708" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="H708" s="5" t="inlineStr">
+      <c r="H708" s="8" t="inlineStr">
         <is>
           <t>Cerrado</t>
         </is>
       </c>
-      <c r="I708" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J708" s="5" t="inlineStr"/>
-      <c r="K708" s="7" t="inlineStr">
+      <c r="I708" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J708" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K708" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.1111/ppl.13097</t>
         </is>
       </c>
-      <c r="L708" s="7" t="inlineStr">
+      <c r="L708" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W3012836007</t>
         </is>
@@ -44104,54 +44157,58 @@
       </c>
     </row>
     <row r="821">
-      <c r="A821" s="5" t="n">
+      <c r="A821" s="8" t="n">
         <v>2018</v>
       </c>
-      <c r="B821" s="6" t="inlineStr">
+      <c r="B821" s="9" t="inlineStr">
         <is>
           <t>The Performance and Potentiality of Monoecious Hemp (Cannabis sativa L.) Cultivars as a Multipurpose Crop</t>
         </is>
       </c>
-      <c r="C821" s="6" t="inlineStr">
+      <c r="C821" s="9" t="inlineStr">
         <is>
           <t>Agronomy</t>
         </is>
       </c>
-      <c r="D821" s="5" t="inlineStr">
+      <c r="D821" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E821" s="6" t="inlineStr">
+      <c r="E821" s="9" t="inlineStr">
         <is>
           <t>Cultivares y tipos de cultivo</t>
         </is>
       </c>
-      <c r="F821" s="6" t="inlineStr">
+      <c r="F821" s="9" t="inlineStr">
         <is>
           <t>Agronomía de grano</t>
         </is>
       </c>
-      <c r="G821" s="5" t="n">
+      <c r="G821" s="8" t="n">
         <v>77</v>
       </c>
-      <c r="H821" s="5" t="inlineStr">
+      <c r="H821" s="8" t="inlineStr">
         <is>
           <t>Abierto (oro/verde)</t>
         </is>
       </c>
-      <c r="I821" s="5" t="inlineStr">
-        <is>
-          <t>Inglés</t>
-        </is>
-      </c>
-      <c r="J821" s="5" t="inlineStr"/>
-      <c r="K821" s="7" t="inlineStr">
+      <c r="I821" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J821" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K821" s="10" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/agronomy8090162</t>
         </is>
       </c>
-      <c r="L821" s="7" t="inlineStr">
+      <c r="L821" s="10" t="inlineStr">
         <is>
           <t>https://openalex.org/W2888070802</t>
         </is>
@@ -51085,8 +51142,840 @@
         </is>
       </c>
     </row>
+    <row r="960">
+      <c r="A960" s="8" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B960" s="9" t="inlineStr">
+        <is>
+          <t>Pathogens and molds affecting production and quality of Cannabis sativa L.</t>
+        </is>
+      </c>
+      <c r="C960" s="9" t="inlineStr">
+        <is>
+          <t>Frontiers in Plant Science</t>
+        </is>
+      </c>
+      <c r="D960" s="8" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="E960" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F960" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G960" s="8" t="n"/>
+      <c r="H960" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I960" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J960" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K960" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fpls.2019.01120</t>
+        </is>
+      </c>
+      <c r="L960" s="10" t="n"/>
+    </row>
+    <row r="961">
+      <c r="A961" s="8" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B961" s="9" t="inlineStr">
+        <is>
+          <t>Diseases of Cannabis sativa caused by diverse Fusarium species</t>
+        </is>
+      </c>
+      <c r="C961" s="9" t="inlineStr">
+        <is>
+          <t>Frontiers in Agronomy</t>
+        </is>
+      </c>
+      <c r="D961" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E961" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F961" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G961" s="8" t="n"/>
+      <c r="H961" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I961" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J961" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K961" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fagro.2021.796062</t>
+        </is>
+      </c>
+      <c r="L961" s="10" t="n"/>
+    </row>
+    <row r="962">
+      <c r="A962" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B962" s="9" t="inlineStr">
+        <is>
+          <t>Pathogenicity and mefenoxam sensitivity of Pythium, Globisporangium, and Fusarium isolates from coconut coir and rockwool in marijuana (Cannabis sativa L.) production</t>
+        </is>
+      </c>
+      <c r="C962" s="9" t="inlineStr">
+        <is>
+          <t>Frontiers in Agronomy</t>
+        </is>
+      </c>
+      <c r="D962" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E962" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F962" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G962" s="8" t="n"/>
+      <c r="H962" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I962" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J962" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K962" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fagro.2021.706138</t>
+        </is>
+      </c>
+      <c r="L962" s="10" t="n"/>
+    </row>
+    <row r="963">
+      <c r="A963" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B963" s="9" t="inlineStr">
+        <is>
+          <t>First insights into the virus and viroid communities in hemp (Cannabis sativa)</t>
+        </is>
+      </c>
+      <c r="C963" s="9" t="inlineStr">
+        <is>
+          <t>Frontiers in Agronomy</t>
+        </is>
+      </c>
+      <c r="D963" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E963" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F963" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G963" s="8" t="n"/>
+      <c r="H963" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I963" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J963" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K963" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fagro.2021.778433</t>
+        </is>
+      </c>
+      <c r="L963" s="10" t="n"/>
+    </row>
+    <row r="964">
+      <c r="A964" s="8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B964" s="9" t="inlineStr">
+        <is>
+          <t>Surveying for potential diseases and abiotic disorders of industrial hemp (Cannabis sativa) production</t>
+        </is>
+      </c>
+      <c r="C964" s="9" t="inlineStr">
+        <is>
+          <t>Plant Health Progress</t>
+        </is>
+      </c>
+      <c r="D964" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E964" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F964" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G964" s="8" t="n"/>
+      <c r="H964" s="8" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="I964" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J964" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K964" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1094/PHP-03-20-0017-RS</t>
+        </is>
+      </c>
+      <c r="L964" s="10" t="n"/>
+    </row>
+    <row r="965">
+      <c r="A965" s="8" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B965" s="9" t="inlineStr">
+        <is>
+          <t>Identificación y caracterización de enfermedades en Cannabis sativa L.</t>
+        </is>
+      </c>
+      <c r="C965" s="9" t="inlineStr">
+        <is>
+          <t>Temas Agrarios</t>
+        </is>
+      </c>
+      <c r="D965" s="8" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="E965" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F965" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G965" s="8" t="n"/>
+      <c r="H965" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I965" s="8" t="inlineStr">
+        <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="J965" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K965" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21897/rta.v27i1.3105</t>
+        </is>
+      </c>
+      <c r="L965" s="10" t="n"/>
+    </row>
+    <row r="966">
+      <c r="A966" s="8" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B966" s="9" t="inlineStr">
+        <is>
+          <t>Developing insect pest management systems for hemp in the United States: A work in progress</t>
+        </is>
+      </c>
+      <c r="C966" s="9" t="inlineStr">
+        <is>
+          <t>Journal of Integrated Pest Management</t>
+        </is>
+      </c>
+      <c r="D966" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E966" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F966" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G966" s="8" t="n"/>
+      <c r="H966" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I966" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J966" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K966" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/jipm/pmz023</t>
+        </is>
+      </c>
+      <c r="L966" s="10" t="n"/>
+    </row>
+    <row r="967">
+      <c r="A967" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B967" s="9" t="inlineStr">
+        <is>
+          <t>Integrated management of pathogens and microbes in Cannabis sativa L. (cannabis) under greenhouse conditions</t>
+        </is>
+      </c>
+      <c r="C967" s="9" t="inlineStr">
+        <is>
+          <t>Plants</t>
+        </is>
+      </c>
+      <c r="D967" s="8" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="E967" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F967" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G967" s="8" t="n"/>
+      <c r="H967" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I967" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J967" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K967" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/plants13060786</t>
+        </is>
+      </c>
+      <c r="L967" s="10" t="n"/>
+    </row>
+    <row r="968">
+      <c r="A968" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B968" s="9" t="inlineStr">
+        <is>
+          <t>Pudrición del cuello de la raíz en pasifloras: Fusarium solani f. sp. passiflorae en sistemas productivos colombianos</t>
+        </is>
+      </c>
+      <c r="C968" s="9" t="inlineStr">
+        <is>
+          <t>Temas Agrarios</t>
+        </is>
+      </c>
+      <c r="D968" s="8" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="E968" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades; Suelo</t>
+        </is>
+      </c>
+      <c r="F968" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G968" s="8" t="n"/>
+      <c r="H968" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I968" s="8" t="inlineStr">
+        <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="J968" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K968" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21897/q15q0254</t>
+        </is>
+      </c>
+      <c r="L968" s="10" t="n"/>
+    </row>
+    <row r="969">
+      <c r="A969" s="8" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B969" s="9" t="inlineStr">
+        <is>
+          <t>Soil health through soil disease suppression: Which strategy from descriptors to indicators?</t>
+        </is>
+      </c>
+      <c r="C969" s="9" t="inlineStr">
+        <is>
+          <t>Soil Biology and Biochemistry</t>
+        </is>
+      </c>
+      <c r="D969" s="8" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E969" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades; Suelo</t>
+        </is>
+      </c>
+      <c r="F969" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G969" s="8" t="n"/>
+      <c r="H969" s="8" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="I969" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J969" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K969" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.soilbio.2006.07.001</t>
+        </is>
+      </c>
+      <c r="L969" s="10" t="n"/>
+    </row>
+    <row r="970">
+      <c r="A970" s="8" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B970" s="9" t="inlineStr">
+        <is>
+          <t>Efecto del cultivo de palma de aceite sobre las propiedades físicas del suelo y su relación con la producción y la pudrición de cogollo</t>
+        </is>
+      </c>
+      <c r="C970" s="9" t="inlineStr">
+        <is>
+          <t>Lámpsakos</t>
+        </is>
+      </c>
+      <c r="D970" s="8" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="E970" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades; Suelo</t>
+        </is>
+      </c>
+      <c r="F970" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G970" s="8" t="n"/>
+      <c r="H970" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I970" s="8" t="inlineStr">
+        <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="J970" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K970" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21501/21454086.2390</t>
+        </is>
+      </c>
+      <c r="L970" s="10" t="n"/>
+    </row>
+    <row r="971">
+      <c r="A971" s="8" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B971" s="9" t="inlineStr">
+        <is>
+          <t>Comparing the yields of organic and conventional agriculture</t>
+        </is>
+      </c>
+      <c r="C971" s="9" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="D971" s="8" t="inlineStr">
+        <is>
+          <t>CA;US</t>
+        </is>
+      </c>
+      <c r="E971" s="9" t="inlineStr">
+        <is>
+          <t>Mercado y economía</t>
+        </is>
+      </c>
+      <c r="F971" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G971" s="8" t="n"/>
+      <c r="H971" s="8" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="I971" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J971" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K971" s="14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/nature11069</t>
+        </is>
+      </c>
+      <c r="L971" s="10" t="n"/>
+    </row>
+    <row r="972">
+      <c r="A972" s="8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B972" s="9" t="inlineStr">
+        <is>
+          <t>2020 on-farm New England hemp pest &amp; disease scouting report</t>
+        </is>
+      </c>
+      <c r="C972" s="9" t="inlineStr">
+        <is>
+          <t>University of Vermont Extension (informe)</t>
+        </is>
+      </c>
+      <c r="D972" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E972" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F972" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G972" s="8" t="n"/>
+      <c r="H972" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I972" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J972" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K972" s="14" t="inlineStr">
+        <is>
+          <t>https://projects.sare.org/wp-content/uploads/2020-Hemp-On-Farm-Scouting-Report-Final.pdf</t>
+        </is>
+      </c>
+      <c r="L972" s="10" t="n"/>
+    </row>
+    <row r="973">
+      <c r="A973" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B973" s="9" t="inlineStr">
+        <is>
+          <t>Economics of producing hemp in NY: Fiber, grain and dual purpose fiber and grain, 2021 budgets</t>
+        </is>
+      </c>
+      <c r="C973" s="9" t="inlineStr">
+        <is>
+          <t>Cornell Cooperative Extension (presupuesto)</t>
+        </is>
+      </c>
+      <c r="D973" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E973" s="9" t="inlineStr">
+        <is>
+          <t>Mercado y economía; Grano y semilla</t>
+        </is>
+      </c>
+      <c r="F973" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G973" s="8" t="n"/>
+      <c r="H973" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I973" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J973" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K973" s="14" t="inlineStr">
+        <is>
+          <t>https://hemp.cals.cornell.edu/files/2021/08/economics-of-industrial-hemp-2021-fiber-grain-dual-purpose-budgets_20210726.pdf</t>
+        </is>
+      </c>
+      <c r="L973" s="10" t="n"/>
+    </row>
+    <row r="974">
+      <c r="A974" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B974" s="9" t="inlineStr">
+        <is>
+          <t>Evaluation of biological insecticides to manage corn earworm in CBD hemp, 2020</t>
+        </is>
+      </c>
+      <c r="C974" s="9" t="inlineStr">
+        <is>
+          <t>Arthropod Management Tests</t>
+        </is>
+      </c>
+      <c r="D974" s="8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E974" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="F974" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G974" s="8" t="n"/>
+      <c r="H974" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I974" s="8" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="J974" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K974" s="14" t="inlineStr">
+        <is>
+          <t>https://hemp.sf.ucdavis.edu/sites/g/files/dgvnsk12601/files/media/documents/Evaluation%20of%20biological%20insecticides%20to%20manage%20corn%20earworm%20in%20CBD%20hemp%2C%202020.pdf</t>
+        </is>
+      </c>
+      <c r="L974" s="10" t="n"/>
+    </row>
+    <row r="975">
+      <c r="A975" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B975" s="9" t="inlineStr">
+        <is>
+          <t>Evaluación del comportamiento de las variedades FT50 y FT70 de Cannabis sativa L. no psicoactivo, bajo condiciones semi controladas y a libre exposición en Campoalegre-Huila</t>
+        </is>
+      </c>
+      <c r="C975" s="9" t="inlineStr">
+        <is>
+          <t>Universidad Nacional Abierta y a Distancia (trabajo de grado)</t>
+        </is>
+      </c>
+      <c r="D975" s="8" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="E975" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades; Trópico y países de baja latitud</t>
+        </is>
+      </c>
+      <c r="F975" s="9" t="inlineStr">
+        <is>
+          <t>Sanidad, MIPE y economía (búsqueda dirigida)</t>
+        </is>
+      </c>
+      <c r="G975" s="8" t="n"/>
+      <c r="H975" s="8" t="inlineStr">
+        <is>
+          <t>Abierto (oro/verde)</t>
+        </is>
+      </c>
+      <c r="I975" s="8" t="inlineStr">
+        <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="J975" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="K975" s="14" t="inlineStr">
+        <is>
+          <t>https://repository.unad.edu.co/jspui/handle/10596/56739</t>
+        </is>
+      </c>
+      <c r="L975" s="10" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L959"/>
+  <autoFilter ref="A1:L975"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -52911,6 +53800,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L958" r:id="rId1821"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K959" r:id="rId1822"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L959" r:id="rId1823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K960" r:id="rId1824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K961" r:id="rId1825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K962" r:id="rId1826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K963" r:id="rId1827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K964" r:id="rId1828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K965" r:id="rId1829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K966" r:id="rId1830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K967" r:id="rId1831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K968" r:id="rId1832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K969" r:id="rId1833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K970" r:id="rId1834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K971" r:id="rId1835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K972" r:id="rId1836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K973" r:id="rId1837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K974" r:id="rId1838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K975" r:id="rId1839"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -53553,6 +54458,14 @@
       <c r="B43" s="13" t="n">
         <v>15</v>
       </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>Sanidad: plagas y enfermedades</t>
+        </is>
+      </c>
+      <c r="E43" s="13" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">

</xml_diff>